<commit_message>
Chèques clients remis (bordereaux CPA) : clients identifiés sur les remises de septembre, registre des remises d'octobre
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XYis4EzVZMNdoYCxmLrRh4
</commit_message>
<xml_diff>
--- a/ETAT_FOURNISSEURS_2026.xlsx
+++ b/ETAT_FOURNISSEURS_2026.xlsx
@@ -2449,7 +2449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:H41"/>
+  <dimension ref="A2:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3026,10 +3026,10 @@
         <v>-738432.49</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>1400000</v>
+        <v>3595116</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>0</v>
+        <v>2433717</v>
       </c>
       <c r="H18" s="8">
         <f>E18+F18-G18</f>
@@ -3494,12 +3494,12 @@
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>FS050</t>
+          <t>FS038</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>CAAR</t>
+          <t>L'ALGERIENNE DES ASSURANCES</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
@@ -3513,13 +3513,13 @@
         </is>
       </c>
       <c r="E32" s="8" t="n">
-        <v>-1934321.62</v>
+        <v>0</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>0</v>
+        <v>5147.25</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>0</v>
+        <v>5147.25</v>
       </c>
       <c r="H32" s="8">
         <f>E32+F32-G32</f>
@@ -3529,12 +3529,12 @@
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>FS066</t>
+          <t>FS050</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>MESBAH IKHLEF</t>
+          <t>CAAR</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
@@ -3548,10 +3548,10 @@
         </is>
       </c>
       <c r="E33" s="8" t="n">
-        <v>-856800</v>
+        <v>-1934321.62</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>1285200</v>
+        <v>0</v>
       </c>
       <c r="G33" s="8" t="n">
         <v>0</v>
@@ -3564,29 +3564,29 @@
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>FI004</t>
+          <t>FS066</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>SARL DPR AXXAM</t>
+          <t>MESBAH IKHLEF</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>40400</t>
+          <t>40130</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>Fournisseurs d'immobilisations</t>
+          <t>FOUR. LOCAUX DE SERVICES</t>
         </is>
       </c>
       <c r="E34" s="8" t="n">
-        <v>-21827400</v>
+        <v>-856800</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>0</v>
+        <v>1285200</v>
       </c>
       <c r="G34" s="8" t="n">
         <v>0</v>
@@ -3599,12 +3599,12 @@
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>FI025</t>
+          <t>FI004</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>SNC RAMTANI&amp;FILS</t>
+          <t>SARL DPR AXXAM</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
@@ -3618,7 +3618,7 @@
         </is>
       </c>
       <c r="E35" s="8" t="n">
-        <v>-81181.96000000001</v>
+        <v>-21827400</v>
       </c>
       <c r="F35" s="8" t="n">
         <v>0</v>
@@ -3634,12 +3634,12 @@
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>FL095</t>
+          <t>FI025</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>SARL BFAHO BENOURATAS</t>
+          <t>SNC RAMTANI&amp;FILS</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
@@ -3653,10 +3653,10 @@
         </is>
       </c>
       <c r="E36" s="8" t="n">
-        <v>0</v>
+        <v>-81181.96000000001</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>4500000</v>
+        <v>0</v>
       </c>
       <c r="G36" s="8" t="n">
         <v>0</v>
@@ -3669,29 +3669,29 @@
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>AF017</t>
+          <t>FL095</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>SARL DPR AXXAM</t>
+          <t>SARL BFAHO BENOURATAS</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>40900</t>
+          <t>40400</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>Fournisseurs débiteurs : avanc</t>
+          <t>Fournisseurs d'immobilisations</t>
         </is>
       </c>
       <c r="E37" s="8" t="n">
-        <v>45350000</v>
+        <v>0</v>
       </c>
       <c r="F37" s="8" t="n">
-        <v>0</v>
+        <v>4500000</v>
       </c>
       <c r="G37" s="8" t="n">
         <v>0</v>
@@ -3704,12 +3704,12 @@
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>AF053</t>
+          <t>AF017</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>TAXE DOMICILIATION BANCAIRE</t>
+          <t>SARL DPR AXXAM</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
@@ -3723,7 +3723,7 @@
         </is>
       </c>
       <c r="E38" s="8" t="n">
-        <v>456100</v>
+        <v>45350000</v>
       </c>
       <c r="F38" s="8" t="n">
         <v>0</v>
@@ -3739,12 +3739,12 @@
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t>AF056</t>
+          <t>AF053</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>KARIM TRANS</t>
+          <t>TAXE DOMICILIATION BANCAIRE</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
@@ -3758,7 +3758,7 @@
         </is>
       </c>
       <c r="E39" s="8" t="n">
-        <v>200000</v>
+        <v>456100</v>
       </c>
       <c r="F39" s="8" t="n">
         <v>0</v>
@@ -3774,12 +3774,12 @@
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>AF059</t>
+          <t>AF056</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>SARL AXECHAN</t>
+          <t>KARIM TRANS</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
@@ -3807,25 +3807,60 @@
       </c>
     </row>
     <row r="41">
-      <c r="B41" s="10" t="inlineStr">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>AF059</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>SARL AXECHAN</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>40900</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>Fournisseurs débiteurs : avanc</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="n">
+        <v>200000</v>
+      </c>
+      <c r="F41" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="8">
+        <f>E41+F41-G41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="10" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E41" s="11">
-        <f>SUM(E4:E40)</f>
-        <v/>
-      </c>
-      <c r="F41" s="11">
-        <f>SUM(F4:F40)</f>
-        <v/>
-      </c>
-      <c r="G41" s="11">
-        <f>SUM(G4:G40)</f>
-        <v/>
-      </c>
-      <c r="H41" s="11">
-        <f>SUM(H4:H40)</f>
+      <c r="E42" s="11">
+        <f>SUM(E4:E41)</f>
+        <v/>
+      </c>
+      <c r="F42" s="11">
+        <f>SUM(F4:F41)</f>
+        <v/>
+      </c>
+      <c r="G42" s="11">
+        <f>SUM(G4:G41)</f>
+        <v/>
+      </c>
+      <c r="H42" s="11">
+        <f>SUM(H4:H41)</f>
         <v/>
       </c>
     </row>

</xml_diff>